<commit_message>
Revise MegaFon connection questionnaire with API credentials and call flow
</commit_message>
<xml_diff>
--- a/3.xlsx
+++ b/3.xlsx
@@ -122,7 +122,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="92" customWidth="1"/>
@@ -132,14 +132,14 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Телефония МегаФон — оставшиеся вопросы</t>
+          <t>Телефония МегаФон — данные для подключения и оставшиеся решения</t>
         </is>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Пожалуйста, заполните правую колонку. Ключи API, пароли и коды доступа сюда не вписывайте — их передают отдельно безопасным способом.</t>
+          <t>Пожалуйста, заполните правую колонку. Если предложенный вариант подходит, напишите «Да». Ключи API, SIP-пароли и коды доступа сюда не вписывайте: их передают отдельно защищённым способом.</t>
         </is>
       </c>
     </row>
@@ -155,114 +155,154 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="72" customHeight="1">
+    <row r="4" ht="84" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>1. Подтвердите, какому из четырёх постоянных сотрудников соответствует каждый внутренний номер 702, 703, 704 и 705. Какие внутренние номера у двух временных аккаунтов стажёров?</t>
+          <t>1. Кто администрирует ВАТС и сможет открыть «Настройки → Интеграция с CRM → Ваша CRM / REST API», включить доступ по API и настроить интеграцию? Укажите имя и способ связи.</t>
         </is>
       </c>
       <c r="B4" s="6"/>
     </row>
-    <row r="5" ht="58" customHeight="1">
+    <row r="5" ht="84" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>2. Стажёры должны получать входящие звонки из общей очереди или им нужны только исходящие? Кто включает и отключает их аккаунты?</t>
+          <t>2. Пришлите адрес Виртуальной АТС из поля «Адрес Виртуальной АТС» (например, https://vats…megapbx.ru), версию/тип API и файл документации REST API из этого раздела. Адрес не является секретом; сам ключ в эту таблицу не вписывайте.</t>
         </is>
       </c>
       <c r="B5" s="6"/>
     </row>
-    <row r="6" ht="72" customHeight="1">
+    <row r="6" ht="84" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>3. Каков установленный тарифом «Мастер коммуникаций» лимит одновременных разговоров? Если его не видно в кабинете, можете запросить подтверждение у МегаФона или приложить скриншот условий тарифа?</t>
+          <t>3. Ключ из поля «Ключ для авторизации в Виртуальной АТС» нужен нашему серверу для исходящих звонков. Кто и каким защищённым способом передаст его нам отдельно от XLSX? Если ключ ещё не создан, кто включит доступ и создаст его?</t>
         </is>
       </c>
       <c r="B6" s="6"/>
     </row>
-    <row r="7" ht="58" customHeight="1">
+    <row r="7" ht="98" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>4. Какой номер должен видеть клиент при исходящем звонке сотрудника из CRM: общий номер компании или личный номер сотрудника?</t>
+          <t>4. Сможет ли администратор ВАТС указать предоставленные нами HTTPS «Адрес вашей CRM» для уведомлений о звонках и отдельный «Ключ для авторизации в вашей CRM»? Подтвердите, что уведомления о входящих, исходящих, завершённых и пропущенных доступны и включаются в вашем кабинете.</t>
         </is>
       </c>
       <c r="B7" s="6"/>
     </row>
-    <row r="8" ht="58" customHeight="1">
+    <row r="8" ht="84" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>5. При новом входящем сколько секунд ждать ответа одного сотрудника перед переводом к следующему? Что делать, если все заняты либо никто не ответил?</t>
+          <t>5. Есть ли ограничение доступа к API по IP-адресу или другие настройки безопасности? Если да, кто добавит IP нашего сервера? Можете прислать скриншоты настроек интеграции с закрытыми ключами и паролями?</t>
         </is>
       </c>
       <c r="B8" s="6"/>
     </row>
-    <row r="9" ht="72" customHeight="1">
+    <row r="9" ht="84" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>6. При повторном звонке, если прежний менеджер занят или отсутствует: переводить клиента другому свободному сотруднику или завершать звонок с обещанием перезвонить? Если перезвонить — в какой срок?</t>
+          <t>6. Подтвердите точное соответствие сотрудников Татьяна, Оксана, Элина, Леонид ↔ внутренние номера 702, 703, 704, 705 и их логины пользователей ВАТС. Какие логины и внутренние номера у двух аккаунтов стажёров?</t>
         </is>
       </c>
       <c r="B9" s="6"/>
     </row>
-    <row r="10" ht="58" customHeight="1">
+    <row r="10" ht="112" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>7. Кому назначать пропущенный первый звонок нового клиента и как уведомлять этого сотрудника: в CRM, по SMS или обоими способами?</t>
+          <t>7. Где сотрудники должны разговаривать: прямо в браузере нашей CRM с гарнитурой или в существующем телефоне/софтфоне, на который АТС сначала звонит после нажатия кнопки «Позвонить» в CRM? Если нужен браузер, попросите поддержку МегаФона подтвердить SIP over WSS/WebRTC для сторонней CRM и дать параметры подключения и отдельные учётные данные каждому оператору (пароли — только защищённым способом).</t>
         </is>
       </c>
       <c r="B10" s="6"/>
     </row>
-    <row r="11" ht="72" customHeight="1">
+    <row r="11" ht="68" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>8. Как сообщать клиенту «Мы перезвоним»: голосовым объявлением во время звонка или отдельным SMS после пропущенного? Если SMS — укажите утверждённый текст и подтвердите согласие на платную отправку.</t>
+          <t>8. Должны ли стажёры принимать входящие из общей очереди или только звонить исходящим? Кто включает и отключает их аккаунты в ВАТС и CRM?</t>
         </is>
       </c>
       <c r="B11" s="6"/>
     </row>
-    <row r="12" ht="72" customHeight="1">
+    <row r="12" ht="112" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>9. Сейчас предупреждения о записи нет. Согласны ли вы включить его перед записываемыми входящими и исходящими звонками? Пришлите утверждённый текст и укажите, кто со стороны компании его согласует.</t>
+          <t>9. Подтвердите единое правило маршрутизации: первый звонок — по очереди; повторный — сначала прежнему менеджеру; если он занят или не ответил, звонок идёт следующему доступному. Сколько секунд ждать одного менеджера? После одного неотвеченного звонка исключать его из очереди на время? Если да, на сколько минут и кто может снять исключение вручную?</t>
         </is>
       </c>
       <c r="B12" s="6"/>
     </row>
-    <row r="13" ht="58" customHeight="1">
+    <row r="13" ht="84" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>10. Кто может прослушивать записи: руководитель, администратор, ответственный по делу? Кому из них разрешить скачивание записи?</t>
+          <t>10. Если никто не ответил или звонок поступил вне рабочего времени, предлагаем проиграть голосом «Мы вам перезвоним» и отметить пропущенный в CRM. Подходит ли это? Укажите рабочие часы, часовой пояс и утверждённый текст объявления.</t>
         </is>
       </c>
       <c r="B13" s="6"/>
     </row>
-    <row r="14" ht="58" customHeight="1">
+    <row r="14" ht="84" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>11. Подтвердите: записи в CRM автоматически удаляются через шесть месяцев со дня звонка. Нужны ли исключения или более раннее удаление по запросу?</t>
+          <t>11. Уведомление о пропущенном делаем внутри CRM с кнопкой «Перезвонить», без SMS и отдельного назначения звонка. Кому показывать уведомление: всем операторам, только последнему говорившему с этим номером или ещё администратору?</t>
         </is>
       </c>
       <c r="B14" s="6"/>
     </row>
-    <row r="15" ht="72" customHeight="1">
+    <row r="15" ht="84" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>12. Полный номер клиента в CRM показывать всем сотрудникам или только тем, кто назначен на обращение/дело, а также руководителю и администратору? Нужно ли фиксировать просмотры номера в журнале?</t>
+          <t>12. Для первого звонка с неизвестного номера: сразу создавать обращение, создавать его только после пропущенного или оставлять звонок в общем журнале до действия сотрудника? Дело автоматически не создаём; подтвердите желаемый вариант.</t>
         </is>
       </c>
       <c r="B15" s="6"/>
     </row>
-    <row r="16" ht="86" customHeight="1">
+    <row r="16" ht="98" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>13. Попросите администратора кабинета или поддержку МегаФона подтвердить две возможности: настройку CRM API и уведомлений о звонках (webhook); звонки прямо в браузере сторонней CRM через SIP over WSS с отдельной учётной записью каждому оператору. Достаточно ответа поддержки или скриншотов без ключей и паролей.</t>
+          <t>13. Где показывать звонки: отдельная общая панель телефонии и история в карточке обращения/клиента или отдельные события внутри чата? У телефонного контакта без сообщений чата пока нет: нужен ли для него пустой чат? Рекомендуем журнал звонков без пустого чата.</t>
         </is>
       </c>
       <c r="B16" s="6"/>
     </row>
-    <row r="17" ht="34" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>Основание: ответы в файле 2.docx. Вопросы об уже подтверждённых услуге ВАТС, общем номере и сроке хранения записей повторно не включены.</t>
+    <row r="17" ht="98" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>14. Если человек позже напишет в мессенджер с тем же номером, связывать его прежние звонки с перепиской и делом по совпадению номера? Подтвердите, что сотрудник должен видеть звонки рядом с чатом/в карточке клиента, а при неоднозначном совпадении связь подтверждается вручную.</t>
+        </is>
+      </c>
+      <c r="B17" s="6"/>
+    </row>
+    <row r="18" ht="98" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>15. Включена ли сейчас опция записи разговоров в ВАТС? Подтвердите у МегаФона, где хранятся записи, каков фактический срок хранения и доступна ли через API ссылка для прослушивания в нашей CRM. Нужно ли хранить отдельную копию в CRM или достаточно записи в ВАТС?</t>
+        </is>
+      </c>
+      <c r="B18" s="6"/>
+    </row>
+    <row r="19" ht="84" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>16. Определите политику записей: какие входящие и исходящие звонки записывать, кто может прослушивать и скачивать записи (включая Софи Николь Левоновну), сколько времени хранить и кто удаляет записи по запросу клиента.</t>
+        </is>
+      </c>
+      <c r="B19" s="6"/>
+    </row>
+    <row r="20" ht="98" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>17. Сейчас голосового предупреждения о записи нет. Подтвердите, что его нужно проигрывать до записываемого разговора, и пришлите утверждённый текст. Кто согласует его и проверит у МегаФона возможность объявления для входящих и исходящих звонков?</t>
+        </is>
+      </c>
+      <c r="B20" s="6"/>
+    </row>
+    <row r="21" ht="84" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>18. Кто сможет вместе с нами провести проверку подключения на тестовом звонке: исходящий из CRM, входящий, пропущенный, уведомление в CRM и запись? Укажите контакт и удобное время. Реальные ключи, SIP-пароли и коды сюда не вписывайте.</t>
+        </is>
+      </c>
+      <c r="B21" s="6"/>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Основание: ответы в 2.docx и раздел МегаФона «Ваша CRM / REST API». Уже подтверждены общий номер компании, последовательная очередь и доступ сотрудников к полному номеру; повторно их не спрашиваем.</t>
         </is>
       </c>
     </row>
@@ -270,7 +310,7 @@
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A22:B22"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>

</xml_diff>

<commit_message>
Name API and webhook tokens explicitly in MegaFon questionnaire
</commit_message>
<xml_diff>
--- a/3.xlsx
+++ b/3.xlsx
@@ -174,7 +174,7 @@
     <row r="6" ht="84" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>3. Ключ из поля «Ключ для авторизации в Виртуальной АТС» нужен нашему серверу для исходящих звонков. Кто и каким защищённым способом передаст его нам отдельно от XLSX? Если ключ ещё не создан, кто включит доступ и создаст его?</t>
+          <t>3. API-токен (ключ из поля «Ключ для авторизации в Виртуальной АТС») нужен нашему серверу для исходящих звонков. Кто и каким защищённым способом передаст его нам отдельно от XLSX? Если токен ещё не создан, кто включит доступ и создаст его?</t>
         </is>
       </c>
       <c r="B6" s="6"/>
@@ -182,7 +182,7 @@
     <row r="7" ht="98" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>4. Сможет ли администратор ВАТС указать предоставленные нами HTTPS «Адрес вашей CRM» для уведомлений о звонках и отдельный «Ключ для авторизации в вашей CRM»? Подтвердите, что уведомления о входящих, исходящих, завершённых и пропущенных доступны и включаются в вашем кабинете.</t>
+          <t>4. Сможет ли администратор ВАТС указать предоставленные нами HTTPS «Адрес вашей CRM» для уведомлений о звонках и отдельный webhook-токен («Ключ для авторизации в вашей CRM»)? Подтвердите, что уведомления о входящих, исходящих, завершённых и пропущенных доступны и включаются в вашем кабинете.</t>
         </is>
       </c>
       <c r="B7" s="6"/>

</xml_diff>

<commit_message>
Reduce MegaFon onboarding to essential PBX setup
</commit_message>
<xml_diff>
--- a/3.xlsx
+++ b/3.xlsx
@@ -122,7 +122,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="92" customWidth="1"/>
@@ -132,14 +132,14 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Телефония МегаФон — данные для подключения и оставшиеся решения</t>
+          <t>МегаФон — минимум для подключения звонков</t>
         </is>
       </c>
     </row>
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Пожалуйста, заполните правую колонку. Если предложенный вариант подходит, напишите «Да». Ключи API, SIP-пароли и коды доступа сюда не вписывайте: их передают отдельно защищённым способом.</t>
+          <t>Пожалуйста, заполните правую колонку. Пароль от кабинета и API-токен передавать в этом файле не нужно. Звонки остаются в ВАТС; CRM показывает события и отправляет команду на исходящий.</t>
         </is>
       </c>
     </row>
@@ -155,42 +155,42 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="84" customHeight="1">
+    <row r="4" ht="98" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>1. Кто администрирует ВАТС и сможет открыть «Настройки → Интеграция с CRM → Ваша CRM / REST API», включить доступ по API и настроить интеграцию? Укажите имя и способ связи.</t>
+          <t>1. Кто сможет на коротком совместном созвоне открыть кабинет ВАТС: «Настройки → Интеграция с CRM → Ваша CRM / REST API», включить доступ по API и скачать инструкцию из этого раздела? Логин и пароль от кабинета нам не нужны; укажите контакт и удобное время.</t>
         </is>
       </c>
       <c r="B4" s="6"/>
     </row>
-    <row r="5" ht="84" customHeight="1">
+    <row r="5" ht="98" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>2. Пришлите адрес Виртуальной АТС из поля «Адрес Виртуальной АТС» (например, https://vats…megapbx.ru), версию/тип API и файл документации REST API из этого раздела. Адрес не является секретом; сам ключ в эту таблицу не вписывайте.</t>
+          <t>2. Для кнопки «Позвонить» нашему серверу нужны только «Адрес Виртуальной АТС» и API-токен («Ключ для авторизации в Виртуальной АТС»). Это отдельный ключ интеграции, не пароль от кабинета. Сможете передать его владельцу проекта защищённым способом? Мы сами внесём его на сервер; в XLSX и переписку токен не вписывайте.</t>
         </is>
       </c>
       <c r="B5" s="6"/>
     </row>
-    <row r="6" ht="84" customHeight="1">
+    <row r="6" ht="98" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>3. API-токен (ключ из поля «Ключ для авторизации в Виртуальной АТС») нужен нашему серверу для исходящих звонков. Кто и каким защищённым способом передаст его нам отдельно от XLSX? Если токен ещё не создан, кто включит доступ и создаст его?</t>
+          <t>3. Сможет ли администратор ВАТС вставить предоставленные нами HTTPS «Адрес вашей CRM» для уведомлений о звонках и отдельный ключ для авторизации в CRM, который мы создадим? Мы подготовим оба значения; нужен только доступ администратора к этой настройке.</t>
         </is>
       </c>
       <c r="B6" s="6"/>
     </row>
-    <row r="7" ht="98" customHeight="1">
+    <row r="7" ht="84" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>4. Сможет ли администратор ВАТС указать предоставленные нами HTTPS «Адрес вашей CRM» для уведомлений о звонках и отдельный webhook-токен («Ключ для авторизации в вашей CRM»)? Подтвердите, что уведомления о входящих, исходящих, завершённых и пропущенных доступны и включаются в вашем кабинете.</t>
+          <t>4. Напишите соответствие четырёх сотрудников Татьяна, Оксана, Элина, Леонид их внутренним номерам 702, 703, 704, 705 и логинам пользователей ВАТС. Логины не являются паролями. Аккаунты стажёров можно подключить позже.</t>
         </is>
       </c>
       <c r="B7" s="6"/>
     </row>
-    <row r="8" ht="84" customHeight="1">
+    <row r="8" ht="98" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>5. Есть ли ограничение доступа к API по IP-адресу или другие настройки безопасности? Если да, кто добавит IP нашего сервера? Можете прислать скриншоты настроек интеграции с закрытыми ключами и паролями?</t>
+          <t>5. Сотрудники продолжат отвечать через свои текущие телефоны или софтфоны? Для исходящего из CRM ВАТС сначала звонит сотруднику, после ответа соединяет с клиентом. Подтвердите, что такой порядок подходит; звонок через браузер CRM не требуется.</t>
         </is>
       </c>
       <c r="B8" s="6"/>
@@ -198,111 +198,15 @@
     <row r="9" ht="84" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>6. Подтвердите точное соответствие сотрудников Татьяна, Оксана, Элина, Леонид ↔ внутренние номера 702, 703, 704, 705 и их логины пользователей ВАТС. Какие логины и внутренние номера у двух аккаунтов стажёров?</t>
+          <t>6. Когда удобно вместе проверить три сценария: исходящий из CRM, входящий с уведомлением поверх интерфейса и пропущенный с кнопкой «Перезвонить»? Укажите контакт и время. Текущую очередь распределения звонков в ВАТС оставляем как есть.</t>
         </is>
       </c>
       <c r="B9" s="6"/>
     </row>
-    <row r="10" ht="112" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>7. Где сотрудники должны разговаривать: прямо в браузере нашей CRM с гарнитурой или в существующем телефоне/софтфоне, на который АТС сначала звонит после нажатия кнопки «Позвонить» в CRM? Если нужен браузер, попросите поддержку МегаФона подтвердить SIP over WSS/WebRTC для сторонней CRM и дать параметры подключения и отдельные учётные данные каждому оператору (пароли — только защищённым способом).</t>
-        </is>
-      </c>
-      <c r="B10" s="6"/>
-    </row>
-    <row r="11" ht="68" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>8. Должны ли стажёры принимать входящие из общей очереди или только звонить исходящим? Кто включает и отключает их аккаунты в ВАТС и CRM?</t>
-        </is>
-      </c>
-      <c r="B11" s="6"/>
-    </row>
-    <row r="12" ht="112" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>9. Подтвердите единое правило маршрутизации: первый звонок — по очереди; повторный — сначала прежнему менеджеру; если он занят или не ответил, звонок идёт следующему доступному. Сколько секунд ждать одного менеджера? После одного неотвеченного звонка исключать его из очереди на время? Если да, на сколько минут и кто может снять исключение вручную?</t>
-        </is>
-      </c>
-      <c r="B12" s="6"/>
-    </row>
-    <row r="13" ht="84" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>10. Если никто не ответил или звонок поступил вне рабочего времени, предлагаем проиграть голосом «Мы вам перезвоним» и отметить пропущенный в CRM. Подходит ли это? Укажите рабочие часы, часовой пояс и утверждённый текст объявления.</t>
-        </is>
-      </c>
-      <c r="B13" s="6"/>
-    </row>
-    <row r="14" ht="84" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>11. Уведомление о пропущенном делаем внутри CRM с кнопкой «Перезвонить», без SMS и отдельного назначения звонка. Кому показывать уведомление: всем операторам, только последнему говорившему с этим номером или ещё администратору?</t>
-        </is>
-      </c>
-      <c r="B14" s="6"/>
-    </row>
-    <row r="15" ht="84" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>12. Для первого звонка с неизвестного номера: сразу создавать обращение, создавать его только после пропущенного или оставлять звонок в общем журнале до действия сотрудника? Дело автоматически не создаём; подтвердите желаемый вариант.</t>
-        </is>
-      </c>
-      <c r="B15" s="6"/>
-    </row>
-    <row r="16" ht="98" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>13. Входящий звонок показываем поверх интерфейса CRM. Где показывать историю: в отдельной общей панели телефонии и карточке обращения/клиента или событиями внутри чата? У телефонного контакта без сообщений чата пока нет: нужен ли пустой чат? Рекомендуем журнал звонков без пустого чата.</t>
-        </is>
-      </c>
-      <c r="B16" s="6"/>
-    </row>
-    <row r="17" ht="98" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>14. Если человек позже напишет в мессенджер с тем же номером, связывать его прежние звонки с перепиской и делом по совпадению номера? Подтвердите, что сотрудник должен видеть звонки рядом с чатом/в карточке клиента, а при неоднозначном совпадении связь подтверждается вручную.</t>
-        </is>
-      </c>
-      <c r="B17" s="6"/>
-    </row>
-    <row r="18" ht="98" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>15. Включена ли сейчас опция записи разговоров в ВАТС? Подтвердите у МегаФона, где хранятся записи, каков фактический срок хранения и доступна ли через API ссылка для прослушивания в нашей CRM. Нужно ли хранить отдельную копию в CRM или достаточно записи в ВАТС?</t>
-        </is>
-      </c>
-      <c r="B18" s="6"/>
-    </row>
-    <row r="19" ht="84" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>16. Определите политику записей: какие входящие и исходящие звонки записывать, кто может прослушивать и скачивать записи (включая Софи Николь Левоновну), сколько времени хранить и кто удаляет записи по запросу клиента.</t>
-        </is>
-      </c>
-      <c r="B19" s="6"/>
-    </row>
-    <row r="20" ht="98" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>17. Сейчас голосового предупреждения о записи нет. Подтвердите, что его нужно проигрывать до записываемого разговора, и пришлите утверждённый текст. Кто согласует его и проверит у МегаФона возможность объявления для входящих и исходящих звонков?</t>
-        </is>
-      </c>
-      <c r="B20" s="6"/>
-    </row>
-    <row r="21" ht="84" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>18. Кто сможет вместе с нами провести проверку подключения на тестовом звонке: исходящий из CRM, входящий, пропущенный, уведомление в CRM и запись? Укажите контакт и удобное время. Реальные ключи, SIP-пароли и коды сюда не вписывайте.</t>
-        </is>
-      </c>
-      <c r="B21" s="6"/>
-    </row>
-    <row r="22" ht="34" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Основание: ответы в 2.docx и раздел МегаФона «Ваша CRM / REST API». Уже подтверждены общий номер компании, последовательная очередь и доступ сотрудников к полному номеру; повторно их не спрашиваем.</t>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Основание: ответы в 2.docx. Общий номер компании и существующую маршрутизацию сохраняем. Записи разговоров, голосовые объявления и связь истории звонков с чатом обсудим после базового подключения.</t>
         </is>
       </c>
     </row>
@@ -310,7 +214,7 @@
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A10:B10"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>

</xml_diff>

<commit_message>
docs: add IFT CRM callback URL to MegaFon questionnaire
</commit_message>
<xml_diff>
--- a/3.xlsx
+++ b/3.xlsx
@@ -156,10 +156,12 @@
       </c>
       <c r="B3" s="6"/>
     </row>
-    <row r="4" ht="112" customHeight="1">
+    <row r="4" ht="136" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2. После того как мы передадим вам HTTPS-адрес API нашей CRM и ключ доступа к этому API для запросов от ВАТС, потребуется в том же разделе ВАТС указать их в полях «Адрес вашей CRM» и «Ключ для авторизации в вашей CRM», затем нажать «Сохранить». Сейчас это делать не нужно. Подтвердите, что у вас будет возможность внести эти значения.</t>
+          <t>2. В личном кабинете ВАТС откройте «Настройки → Интеграция с CRM → Ваша CRM / REST API». В поле «Адрес вашей CRM» вставьте адрес тестового контура:
+https://ift.135.106.181.236.nip.io/api/v1/integrations/webhooks/megafon
+В поле «Ключ для авторизации в вашей CRM» вставьте отдельный ключ, который мы передадим по защищённому каналу. Нажмите «Сохранить» и сообщите нам.</t>
         </is>
       </c>
       <c r="B4" s="6"/>

</xml_diff>